<commit_message>
New Qubex ProLogic STD 7000 BR08-T/PL 7040 STDCRT IO Pics
</commit_message>
<xml_diff>
--- a/_Qubex_Disk_Analyzer/Master_BOM.xlsx
+++ b/_Qubex_Disk_Analyzer/Master_BOM.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\_DOCUMENTS\_Retro_Computing_Stuff\__MY_Vintage_Equipment\_Qubex_Disk_Analyzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD6378E-AE71-4BF8-BEBF-47E6ADB9CFF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B41A1F-D3D5-40B6-B433-3E2A91F973CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2790" yWindow="315" windowWidth="18000" windowHeight="9480" xr2:uid="{6AB15EB7-D830-4F52-B1A7-6BE594ACCF47}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{6AB15EB7-D830-4F52-B1A7-6BE594ACCF47}"/>
   </bookViews>
   <sheets>
-    <sheet name="IO RAM Expansion Board" sheetId="1" r:id="rId1"/>
+    <sheet name="Cubit 7040 STDCRT" sheetId="2" r:id="rId1"/>
+    <sheet name="Cubit 7041 RAM Expansion" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="91">
   <si>
     <t>Synertek</t>
   </si>
@@ -64,6 +65,240 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>Signetics</t>
+  </si>
+  <si>
+    <t>Intel</t>
+  </si>
+  <si>
+    <t>NEC</t>
+  </si>
+  <si>
+    <t>D2716</t>
+  </si>
+  <si>
+    <t>10uf 16v</t>
+  </si>
+  <si>
+    <t>Electrolytic Cap</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>U4</t>
+  </si>
+  <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>U11</t>
+  </si>
+  <si>
+    <t>U12</t>
+  </si>
+  <si>
+    <t>U8</t>
+  </si>
+  <si>
+    <t>U6</t>
+  </si>
+  <si>
+    <t>U7</t>
+  </si>
+  <si>
+    <t>U9</t>
+  </si>
+  <si>
+    <t>U10</t>
+  </si>
+  <si>
+    <t>Board Part #/Model</t>
+  </si>
+  <si>
+    <t>7040 (300882)</t>
+  </si>
+  <si>
+    <t>Cubit Inc. 1982</t>
+  </si>
+  <si>
+    <t>National Semiconductor</t>
+  </si>
+  <si>
+    <t>DM74LS221N</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>74LS166N</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>F (Indonesia)</t>
+  </si>
+  <si>
+    <t>74LS378PC</t>
+  </si>
+  <si>
+    <t>P8275</t>
+  </si>
+  <si>
+    <t>AMD</t>
+  </si>
+  <si>
+    <t>8255A</t>
+  </si>
+  <si>
+    <t>8085AH</t>
+  </si>
+  <si>
+    <t>D2716D</t>
+  </si>
+  <si>
+    <t>SN74LS373N</t>
+  </si>
+  <si>
+    <t>74LS02PC</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>6.144Mhz</t>
+  </si>
+  <si>
+    <t>F (Singapore)</t>
+  </si>
+  <si>
+    <t>U20</t>
+  </si>
+  <si>
+    <t>U15</t>
+  </si>
+  <si>
+    <t>U18</t>
+  </si>
+  <si>
+    <t>U19</t>
+  </si>
+  <si>
+    <t>U24</t>
+  </si>
+  <si>
+    <t>U25</t>
+  </si>
+  <si>
+    <t>U26</t>
+  </si>
+  <si>
+    <t>U27</t>
+  </si>
+  <si>
+    <t>U23</t>
+  </si>
+  <si>
+    <t>U22</t>
+  </si>
+  <si>
+    <t>SN74LS166N</t>
+  </si>
+  <si>
+    <t>U16</t>
+  </si>
+  <si>
+    <t>U17</t>
+  </si>
+  <si>
+    <t>EMPTY SOCKET</t>
+  </si>
+  <si>
+    <t>Monolithic Memory MMI</t>
+  </si>
+  <si>
+    <t>DM74LS74AN</t>
+  </si>
+  <si>
+    <t>U14</t>
+  </si>
+  <si>
+    <t>74LS02N</t>
+  </si>
+  <si>
+    <t>U13</t>
+  </si>
+  <si>
+    <t>Motorola</t>
+  </si>
+  <si>
+    <t>74LS04N</t>
+  </si>
+  <si>
+    <t>DM74LS32N</t>
+  </si>
+  <si>
+    <t>74LS138PC</t>
+  </si>
+  <si>
+    <t>74S135PC</t>
+  </si>
+  <si>
+    <t>74LS12N</t>
+  </si>
+  <si>
+    <t>74LS10N</t>
+  </si>
+  <si>
+    <t>74LS139PC</t>
+  </si>
+  <si>
+    <t>SN74LS244N</t>
+  </si>
+  <si>
+    <t>74LS245N</t>
+  </si>
+  <si>
+    <t>U21</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>12.48Mhz</t>
+  </si>
+  <si>
+    <t>MF Electronics</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>R8</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>X104 (100k?)</t>
+  </si>
+  <si>
+    <t>Multi-turn trip pot</t>
   </si>
 </sst>
 </file>
@@ -427,8 +662,568 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEC0236-51E9-440B-A2E8-3EBAC6B02E1F}">
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="29.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" style="1" customWidth="1"/>
+    <col min="3" max="4" width="9.140625" style="1"/>
+    <col min="5" max="5" width="11.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="27.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="1">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1">
+        <v>8219</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="1">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1">
+        <v>8227</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="1">
+        <v>16</v>
+      </c>
+      <c r="E8" s="1">
+        <v>8101</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="1">
+        <v>14</v>
+      </c>
+      <c r="E9" s="1">
+        <v>8203</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="1">
+        <v>14</v>
+      </c>
+      <c r="E10" s="1">
+        <v>7850</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="1">
+        <v>14</v>
+      </c>
+      <c r="E11" s="1">
+        <v>7945</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="1">
+        <v>16</v>
+      </c>
+      <c r="E12" s="1">
+        <v>7744</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="1">
+        <v>40</v>
+      </c>
+      <c r="E13" s="1">
+        <v>8107</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="1">
+        <v>40</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="1">
+        <v>14</v>
+      </c>
+      <c r="E15" s="1">
+        <v>8101</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="1">
+        <v>14</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="1">
+        <v>14</v>
+      </c>
+      <c r="E17" s="1">
+        <v>8008</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="1">
+        <v>14</v>
+      </c>
+      <c r="E18" s="1">
+        <v>8033</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="1">
+        <v>14</v>
+      </c>
+      <c r="E19" s="1">
+        <v>8203</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="1">
+        <v>28</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="1">
+        <v>24</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="1">
+        <v>24</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="1">
+        <v>40</v>
+      </c>
+      <c r="E23" s="1">
+        <v>8107</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="1">
+        <v>40</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="1">
+        <v>24</v>
+      </c>
+      <c r="E25" s="1">
+        <v>8221</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D26" s="1">
+        <v>14</v>
+      </c>
+      <c r="E26" s="1">
+        <v>7948</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="1">
+        <v>8009</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="1">
+        <v>20</v>
+      </c>
+      <c r="E28" s="1">
+        <v>8221</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="1">
+        <v>16</v>
+      </c>
+      <c r="E29" s="1">
+        <v>8040</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="1">
+        <v>16</v>
+      </c>
+      <c r="E30" s="1">
+        <v>8009</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="1">
+        <v>16</v>
+      </c>
+      <c r="E31" s="1">
+        <v>7937</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="1">
+        <v>16</v>
+      </c>
+      <c r="E32" s="1">
+        <v>7937</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="1">
+        <v>8230</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G35" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G36" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G37" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G38" t="s">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A9:F14">
+    <sortCondition ref="F9:F14"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91C527C7-4210-49AE-A95E-3FDBC1725346}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" style="1" customWidth="1"/>
@@ -470,11 +1265,17 @@
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1">
-        <v>8251</v>
-      </c>
       <c r="D2" s="1">
         <v>24</v>
+      </c>
+      <c r="E2" s="1">
+        <v>8251</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -484,11 +1285,17 @@
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1">
-        <v>8251</v>
-      </c>
       <c r="D3" s="1">
         <v>24</v>
+      </c>
+      <c r="E3" s="1">
+        <v>8251</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -498,11 +1305,17 @@
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="1">
-        <v>8251</v>
-      </c>
       <c r="D4" s="1">
         <v>24</v>
+      </c>
+      <c r="E4" s="1">
+        <v>8251</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -512,14 +1325,23 @@
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="1">
-        <v>8251</v>
-      </c>
       <c r="D5" s="1">
         <v>24</v>
       </c>
+      <c r="E5" s="1">
+        <v>8251</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
@@ -529,8 +1351,14 @@
       <c r="E6" s="1">
         <v>8232</v>
       </c>
+      <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -540,8 +1368,14 @@
       <c r="E7" s="1">
         <v>8038</v>
       </c>
+      <c r="F7" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
@@ -551,16 +1385,89 @@
       <c r="E8" s="1">
         <v>8038</v>
       </c>
+      <c r="F8" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="1">
         <v>28</v>
       </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="G9" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="1">
+        <v>24</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="1">
+        <v>24</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="1">
+        <v>24</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="1">
+        <v>24</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>